<commit_message>
Daily slate 2026-05-15 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-13.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-13.xlsx
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -645,13 +645,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3424</v>
+        <v>3425</v>
       </c>
       <c r="E8" t="n">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F8" t="n">
-        <v>2899</v>
+        <v>2901</v>
       </c>
       <c r="G8" t="n">
         <v>15.3</v>
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="E10" t="n">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F10" t="n">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G10" t="n">
-        <v>59.4</v>
+        <v>59.3</v>
       </c>
     </row>
     <row r="11">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E15" t="n">
         <v>7</v>
       </c>
       <c r="F15" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G15" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2079</v>
+        <v>2098</v>
       </c>
       <c r="E17" t="n">
         <v>454</v>
       </c>
       <c r="F17" t="n">
-        <v>1625</v>
+        <v>1644</v>
       </c>
       <c r="G17" t="n">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
     </row>
   </sheetData>
@@ -1236,7 +1236,7 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>15</v>
+        <v>14.7</v>
       </c>
       <c r="Y3" t="n">
         <v>421</v>
@@ -1483,10 +1483,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>59.4</v>
+        <v>59.3</v>
       </c>
       <c r="C7" t="n">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D7" t="n">
         <v>64.2</v>
@@ -1513,10 +1513,10 @@
         <v>69</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="N7" t="n">
         <v>29.4</v>
@@ -1525,10 +1525,10 @@
         <v>17</v>
       </c>
       <c r="P7" t="n">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>2079</v>
+        <v>2098</v>
       </c>
       <c r="R7" t="n">
         <v>50.9</v>
@@ -1543,16 +1543,16 @@
         <v>20</v>
       </c>
       <c r="V7" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="W7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X7" t="n">
         <v>15.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>3424</v>
+        <v>3425</v>
       </c>
       <c r="Z7" t="n">
         <v>70.59999999999999</v>

</xml_diff>